<commit_message>
Updated Register Data in Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324D4FBA-1DDD-4E18-A7FB-76C96524A489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C6EC81-4D9C-40DD-B3D3-9ADB7FDA3C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad163@gmail.com</t>
+    <t>bad173@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added new Datas in Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DC2DE5-51A6-4CB9-B03E-86BD0BEBCFFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A419B94E-2DE2-47B6-ADA9-93B72E845AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad134@gmail.com</t>
+    <t>bad114@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Made changes for Parallel Execution
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A419B94E-2DE2-47B6-ADA9-93B72E845AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90A9EA2-E191-4CAC-86A4-E8094B2886B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad114@gmail.com</t>
+    <t>bad232@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Register Data Changes in Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90A9EA2-E191-4CAC-86A4-E8094B2886B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B528F07-C34B-4057-9EFF-22BBD2D0DA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3984" yWindow="1752" windowWidth="17280" windowHeight="9948" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registerVData" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>bad232@gmail.com</t>
+    <t>tilo007@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added new Test data in Register Excel File
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJavaAutomationProject\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69282C3D-1419-40D2-8D7F-2109DFF260C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A6F20C0-C7AF-49E3-AA26-3B9474CCAFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>tilo010@gmail.com</t>
+    <t>tilo011@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updated the parallel execution
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D86394EF-466C-4038-AD24-B0F3A615140E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Automation-Project-main\E-Commerce Lambdatest\src\test\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0ACF47F-658C-40CB-A8F9-5364B18ED086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +16,6 @@
     <sheet name="registerVData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -53,7 +57,7 @@
     <t>bad100</t>
   </si>
   <si>
-    <t>tilo0jb13@gmail.com</t>
+    <t>dik31@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updated Excel Data on Register Details
</commit_message>
<xml_diff>
--- a/src/test/resources/register_data.xlsx
+++ b/src/test/resources/register_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Automation-Project-main\E-Commerce Lambdatest\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java_Selenium_Project_cucumber\Automation-Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF626B9-D916-4E16-A6C6-E887CB4CAEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1630555D-41DB-48F1-A895-808ACCF18055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registerVData" sheetId="1" r:id="rId1"/>
@@ -51,10 +51,10 @@
     <t>Adhi</t>
   </si>
   <si>
-    <t>bad100</t>
-  </si>
-  <si>
-    <t>fiz12z5@gmail.com</t>
+    <t>farruk125@gmail.com</t>
+  </si>
+  <si>
+    <t>baggy100</t>
   </si>
 </sst>
 </file>
@@ -423,16 +423,16 @@
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2">
         <v>1209348756</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>